<commit_message>
updated Contractor Databse, cleaned up data folder
</commit_message>
<xml_diff>
--- a/server/src/data/ContractorDatabase.xlsx
+++ b/server/src/data/ContractorDatabase.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Projects\forestry_company_database\server\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9596A6A-D1EE-4118-9553-41B11EB3F257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53EFE6D-2DE7-4CF0-8278-628263D9E280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="106">
   <si>
     <t>Contractors name</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t>250-305-6326</t>
+  </si>
+  <si>
+    <t>Ponsse Scorpion (harvester), Ponsse Bear (harvester), Eltec 227 with a Ponsse H8 head (tracked harvester), Eltec 277 with a Ponsse H8 head (tracked harvester), Ponsse Elephant King (forwarder), Ponsse Buffalo King (forwarder), John Deere 1910 (forwarder)</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1258,9 @@
       <c r="J16" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="K16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
@@ -1297,15 +1302,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x010100D5593F09D3A6E34AADF527B1A86CF6BC" ma:contentTypeVersion="11" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="a37b25d9638c04ca7dacd8a7464e4584">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="a5da3473-866d-4fcf-ba99-61417476e810" xmlns:ns4="5abbb7ee-d7fd-4112-9453-4da709f8202f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="772756a5ea4411630b2aee7b9d37809d" ns3:_="" ns4:_="">
     <xsd:import namespace="a5da3473-866d-4fcf-ba99-61417476e810"/>
@@ -1514,6 +1510,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1523,14 +1528,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F1BE107-753B-40F0-9FDC-4B5607A9EE69}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E15B24C3-5AF3-4FFA-90EF-8FE61C1C67E3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1545,6 +1542,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F1BE107-753B-40F0-9FDC-4B5607A9EE69}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>